<commit_message>
fixed the issue of multiple repeaters replying WOR-ACK to the same ED despite hearing each other
</commit_message>
<xml_diff>
--- a/Tests/representative_network_1_sim_outputs.xlsx
+++ b/Tests/representative_network_1_sim_outputs.xlsx
@@ -2698,7 +2698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N332"/>
+  <dimension ref="A1:N371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" min="3" max="3"/>
@@ -16936,6 +16936,1917 @@
         <v>3178.862301357323</v>
       </c>
     </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>1</v>
+      </c>
+      <c r="B333" t="n">
+        <v>51</v>
+      </c>
+      <c r="C333" t="n">
+        <v>4</v>
+      </c>
+      <c r="D333" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E333" t="n">
+        <v>1</v>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G333" t="n">
+        <v>1</v>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I333" t="n">
+        <v>58.61480498127639</v>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K333" t="n">
+        <v>58.61480498127639</v>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M333" t="n">
+        <v>58.61480498127639</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>1</v>
+      </c>
+      <c r="B334" t="n">
+        <v>51</v>
+      </c>
+      <c r="C334" t="n">
+        <v>4</v>
+      </c>
+      <c r="D334" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E334" t="n">
+        <v>1</v>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G334" t="n">
+        <v>1</v>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I334" t="n">
+        <v>10725.33866530866</v>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K334" t="n">
+        <v>10725.33866530866</v>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M334" t="n">
+        <v>10725.33866530866</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>1</v>
+      </c>
+      <c r="B335" t="n">
+        <v>51</v>
+      </c>
+      <c r="C335" t="n">
+        <v>4</v>
+      </c>
+      <c r="D335" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E335" t="n">
+        <v>1</v>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G335" t="n">
+        <v>1</v>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I335" t="n">
+        <v>3127.101051932666</v>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K335" t="n">
+        <v>3127.101051932666</v>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M335" t="n">
+        <v>3127.101051932666</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>1</v>
+      </c>
+      <c r="B336" t="n">
+        <v>51</v>
+      </c>
+      <c r="C336" t="n">
+        <v>4</v>
+      </c>
+      <c r="D336" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E336" t="n">
+        <v>3</v>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G336" t="n">
+        <v>1</v>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I336" t="n">
+        <v>3817.46713262094</v>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K336" t="n">
+        <v>3107.672593640396</v>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M336" t="n">
+        <v>4178.943745661178</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>1</v>
+      </c>
+      <c r="B337" t="n">
+        <v>51</v>
+      </c>
+      <c r="C337" t="n">
+        <v>4</v>
+      </c>
+      <c r="D337" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E337" t="n">
+        <v>1</v>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G337" t="n">
+        <v>1</v>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I337" t="n">
+        <v>10134.51963094692</v>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K337" t="n">
+        <v>10134.51963094692</v>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M337" t="n">
+        <v>10134.51963094692</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>1</v>
+      </c>
+      <c r="B338" t="n">
+        <v>51</v>
+      </c>
+      <c r="C338" t="n">
+        <v>4</v>
+      </c>
+      <c r="D338" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E338" t="n">
+        <v>1</v>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G338" t="n">
+        <v>1</v>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I338" t="n">
+        <v>9757.470952335498</v>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K338" t="n">
+        <v>9757.470952335498</v>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M338" t="n">
+        <v>9757.470952335498</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>1</v>
+      </c>
+      <c r="B339" t="n">
+        <v>51</v>
+      </c>
+      <c r="C339" t="n">
+        <v>4</v>
+      </c>
+      <c r="D339" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E339" t="n">
+        <v>1</v>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G339" t="n">
+        <v>1</v>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I339" t="n">
+        <v>3154.562645594749</v>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K339" t="n">
+        <v>3154.562645594749</v>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M339" t="n">
+        <v>3154.562645594749</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>1</v>
+      </c>
+      <c r="B340" t="n">
+        <v>51</v>
+      </c>
+      <c r="C340" t="n">
+        <v>4</v>
+      </c>
+      <c r="D340" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E340" t="n">
+        <v>1</v>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G340" t="n">
+        <v>1</v>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I340" t="n">
+        <v>3108.793945197482</v>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K340" t="n">
+        <v>3108.793945197482</v>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M340" t="n">
+        <v>3108.793945197482</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>1</v>
+      </c>
+      <c r="B341" t="n">
+        <v>51</v>
+      </c>
+      <c r="C341" t="n">
+        <v>4</v>
+      </c>
+      <c r="D341" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E341" t="n">
+        <v>1</v>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G341" t="n">
+        <v>1</v>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I341" t="n">
+        <v>1059.496784052579</v>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K341" t="n">
+        <v>1059.496784052579</v>
+      </c>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M341" t="n">
+        <v>1059.496784052579</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>1</v>
+      </c>
+      <c r="B342" t="n">
+        <v>51</v>
+      </c>
+      <c r="C342" t="n">
+        <v>4</v>
+      </c>
+      <c r="D342" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E342" t="n">
+        <v>5</v>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G342" t="n">
+        <v>1</v>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I342" t="n">
+        <v>3822.3178409165</v>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K342" t="n">
+        <v>3127.97276435711</v>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M342" t="n">
+        <v>4151.099299124442</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="n">
+        <v>1</v>
+      </c>
+      <c r="B343" t="n">
+        <v>51</v>
+      </c>
+      <c r="C343" t="n">
+        <v>4</v>
+      </c>
+      <c r="D343" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E343" t="n">
+        <v>5</v>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G343" t="n">
+        <v>1</v>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I343" t="n">
+        <v>3664.424253222183</v>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K343" t="n">
+        <v>2141.904956761864</v>
+      </c>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M343" t="n">
+        <v>4155.159989645705</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="n">
+        <v>1</v>
+      </c>
+      <c r="B344" t="n">
+        <v>51</v>
+      </c>
+      <c r="C344" t="n">
+        <v>4</v>
+      </c>
+      <c r="D344" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E344" t="n">
+        <v>5</v>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G344" t="n">
+        <v>1</v>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I344" t="n">
+        <v>3744.613384033647</v>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K344" t="n">
+        <v>2166.315523772035</v>
+      </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M344" t="n">
+        <v>5148.411615606397</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="n">
+        <v>1</v>
+      </c>
+      <c r="B345" t="n">
+        <v>51</v>
+      </c>
+      <c r="C345" t="n">
+        <v>4</v>
+      </c>
+      <c r="D345" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E345" t="n">
+        <v>5</v>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G345" t="n">
+        <v>1</v>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I345" t="n">
+        <v>4289.404266266618</v>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K345" t="n">
+        <v>3113.111970863771</v>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M345" t="n">
+        <v>6247.118597372435</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="n">
+        <v>1</v>
+      </c>
+      <c r="B346" t="n">
+        <v>51</v>
+      </c>
+      <c r="C346" t="n">
+        <v>4</v>
+      </c>
+      <c r="D346" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E346" t="n">
+        <v>5</v>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G346" t="n">
+        <v>1</v>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I346" t="n">
+        <v>5232.711353173479</v>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K346" t="n">
+        <v>2081.399946427904</v>
+      </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M346" t="n">
+        <v>10159.52191505954</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="n">
+        <v>1</v>
+      </c>
+      <c r="B347" t="n">
+        <v>51</v>
+      </c>
+      <c r="C347" t="n">
+        <v>4</v>
+      </c>
+      <c r="D347" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E347" t="n">
+        <v>5</v>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G347" t="n">
+        <v>1</v>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I347" t="n">
+        <v>3393.032398927957</v>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K347" t="n">
+        <v>2110.52681506332</v>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M347" t="n">
+        <v>4421.279437793419</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>1</v>
+      </c>
+      <c r="B348" t="n">
+        <v>51</v>
+      </c>
+      <c r="C348" t="n">
+        <v>4</v>
+      </c>
+      <c r="D348" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E348" t="n">
+        <v>5</v>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G348" t="n">
+        <v>1</v>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I348" t="n">
+        <v>2876.951388835162</v>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K348" t="n">
+        <v>2047.728294204921</v>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M348" t="n">
+        <v>4090.593256166205</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="n">
+        <v>1</v>
+      </c>
+      <c r="B349" t="n">
+        <v>51</v>
+      </c>
+      <c r="C349" t="n">
+        <v>4</v>
+      </c>
+      <c r="D349" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E349" t="n">
+        <v>5</v>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G349" t="n">
+        <v>1</v>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I349" t="n">
+        <v>1861.909936257079</v>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K349" t="n">
+        <v>42.83447280153632</v>
+      </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M349" t="n">
+        <v>3074.131317925639</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="n">
+        <v>1</v>
+      </c>
+      <c r="B350" t="n">
+        <v>51</v>
+      </c>
+      <c r="C350" t="n">
+        <v>4</v>
+      </c>
+      <c r="D350" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E350" t="n">
+        <v>5</v>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G350" t="n">
+        <v>1</v>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I350" t="n">
+        <v>3288.954653291684</v>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K350" t="n">
+        <v>2065.242273322772</v>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M350" t="n">
+        <v>4126.484229970723</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>1</v>
+      </c>
+      <c r="B351" t="n">
+        <v>17</v>
+      </c>
+      <c r="C351" t="n">
+        <v>3</v>
+      </c>
+      <c r="D351" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="E351" t="n">
+        <v>5</v>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G351" t="n">
+        <v>1</v>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I351" t="n">
+        <v>2079.128513267732</v>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K351" t="n">
+        <v>1071.199210533872</v>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M351" t="n">
+        <v>3139.44299081825</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="n">
+        <v>1</v>
+      </c>
+      <c r="B352" t="n">
+        <v>17</v>
+      </c>
+      <c r="C352" t="n">
+        <v>3</v>
+      </c>
+      <c r="D352" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="E352" t="n">
+        <v>50</v>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G352" t="n">
+        <v>1</v>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I352" t="n">
+        <v>2329.586926977969</v>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K352" t="n">
+        <v>33.1211746763438</v>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M352" t="n">
+        <v>4109.210127131082</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>1</v>
+      </c>
+      <c r="B353" t="n">
+        <v>17</v>
+      </c>
+      <c r="C353" t="n">
+        <v>3</v>
+      </c>
+      <c r="D353" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="E353" t="n">
+        <v>50</v>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G353" t="n">
+        <v>1</v>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I353" t="n">
+        <v>2021.476221156154</v>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K353" t="n">
+        <v>32.22097335197031</v>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M353" t="n">
+        <v>4150.298076206818</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="n">
+        <v>1</v>
+      </c>
+      <c r="B354" t="n">
+        <v>17</v>
+      </c>
+      <c r="C354" t="n">
+        <v>3</v>
+      </c>
+      <c r="D354" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="E354" t="n">
+        <v>100</v>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G354" t="n">
+        <v>1</v>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I354" t="n">
+        <v>2075.31295470349</v>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K354" t="n">
+        <v>32.18667261302471</v>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M354" t="n">
+        <v>4122.799322558567</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="n">
+        <v>1</v>
+      </c>
+      <c r="B355" t="n">
+        <v>17</v>
+      </c>
+      <c r="C355" t="n">
+        <v>3</v>
+      </c>
+      <c r="D355" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="E355" t="n">
+        <v>5</v>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G355" t="n">
+        <v>1</v>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I355" t="n">
+        <v>2068.84601060024</v>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K355" t="n">
+        <v>2062.952625455102</v>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M355" t="n">
+        <v>2074.747552380664</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="n">
+        <v>1</v>
+      </c>
+      <c r="B356" t="n">
+        <v>17</v>
+      </c>
+      <c r="C356" t="n">
+        <v>3</v>
+      </c>
+      <c r="D356" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="E356" t="n">
+        <v>5</v>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G356" t="n">
+        <v>1</v>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I356" t="n">
+        <v>1651.18833288484</v>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K356" t="n">
+        <v>42.76433212403208</v>
+      </c>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M356" t="n">
+        <v>4065.408612984349</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="n">
+        <v>1</v>
+      </c>
+      <c r="B357" t="n">
+        <v>17</v>
+      </c>
+      <c r="C357" t="n">
+        <v>3</v>
+      </c>
+      <c r="D357" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="E357" t="n">
+        <v>500</v>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G357" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I357" t="n">
+        <v>2743.334020974688</v>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K357" t="n">
+        <v>31.97082609310746</v>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M357" t="n">
+        <v>26259.22007218748</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="n">
+        <v>1</v>
+      </c>
+      <c r="B358" t="n">
+        <v>17</v>
+      </c>
+      <c r="C358" t="n">
+        <v>3</v>
+      </c>
+      <c r="D358" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="E358" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G358" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I358" t="n">
+        <v>2878.974056583224</v>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K358" t="n">
+        <v>32.0190721154213</v>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M358" t="n">
+        <v>25996.47737404704</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="n">
+        <v>1</v>
+      </c>
+      <c r="B359" t="n">
+        <v>17</v>
+      </c>
+      <c r="C359" t="n">
+        <v>3</v>
+      </c>
+      <c r="D359" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E359" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G359" t="n">
+        <v>0.903</v>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I359" t="n">
+        <v>3288.354470799401</v>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K359" t="n">
+        <v>31.89861626178026</v>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M359" t="n">
+        <v>29988.6796085618</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="n">
+        <v>1</v>
+      </c>
+      <c r="B360" t="n">
+        <v>17</v>
+      </c>
+      <c r="C360" t="n">
+        <v>3</v>
+      </c>
+      <c r="D360" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E360" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G360" t="n">
+        <v>0.948</v>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I360" t="n">
+        <v>2539.75145829734</v>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K360" t="n">
+        <v>31.87001639278606</v>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M360" t="n">
+        <v>17056.38656454533</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="n">
+        <v>1</v>
+      </c>
+      <c r="B361" t="n">
+        <v>17</v>
+      </c>
+      <c r="C361" t="n">
+        <v>3</v>
+      </c>
+      <c r="D361" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E361" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G361" t="n">
+        <v>0.922</v>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I361" t="n">
+        <v>2501.310926654074</v>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K361" t="n">
+        <v>31.87104577943683</v>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M361" t="n">
+        <v>24300.27257366944</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>1</v>
+      </c>
+      <c r="B362" t="n">
+        <v>17</v>
+      </c>
+      <c r="C362" t="n">
+        <v>3</v>
+      </c>
+      <c r="D362" t="n">
+        <v>36000</v>
+      </c>
+      <c r="E362" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G362" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I362" t="n">
+        <v>8125.112571291661</v>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K362" t="n">
+        <v>31.96342869265936</v>
+      </c>
+      <c r="L362" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M362" t="n">
+        <v>62642.44422572944</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>1</v>
+      </c>
+      <c r="B363" t="n">
+        <v>17</v>
+      </c>
+      <c r="C363" t="n">
+        <v>3</v>
+      </c>
+      <c r="D363" t="n">
+        <v>36000</v>
+      </c>
+      <c r="E363" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G363" t="n">
+        <v>0.5620000000000001</v>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I363" t="n">
+        <v>9518.371068568957</v>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K363" t="n">
+        <v>31.99394500366179</v>
+      </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M363" t="n">
+        <v>92774.10036211228</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>1</v>
+      </c>
+      <c r="B364" t="n">
+        <v>17</v>
+      </c>
+      <c r="C364" t="n">
+        <v>3</v>
+      </c>
+      <c r="D364" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E364" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G364" t="n">
+        <v>0.9389999999999999</v>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I364" t="n">
+        <v>2378.768841339481</v>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K364" t="n">
+        <v>31.86684214510024</v>
+      </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M364" t="n">
+        <v>16520.49515233934</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>1</v>
+      </c>
+      <c r="B365" t="n">
+        <v>17</v>
+      </c>
+      <c r="C365" t="n">
+        <v>3</v>
+      </c>
+      <c r="D365" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E365" t="n">
+        <v>500</v>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G365" t="n">
+        <v>0.9419999999999999</v>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I365" t="n">
+        <v>2325.143455863505</v>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K365" t="n">
+        <v>31.88181386119686</v>
+      </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M365" t="n">
+        <v>17614.01453115046</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>1</v>
+      </c>
+      <c r="B366" t="n">
+        <v>51</v>
+      </c>
+      <c r="C366" t="n">
+        <v>4</v>
+      </c>
+      <c r="D366" t="n">
+        <v>36000000</v>
+      </c>
+      <c r="E366" t="n">
+        <v>5</v>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G366" t="n">
+        <v>1</v>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I366" t="n">
+        <v>3889.472682507243</v>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K366" t="n">
+        <v>2054.757705111057</v>
+      </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M366" t="n">
+        <v>6136.013922041282</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>1</v>
+      </c>
+      <c r="B367" t="n">
+        <v>17</v>
+      </c>
+      <c r="C367" t="n">
+        <v>3</v>
+      </c>
+      <c r="D367" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E367" t="n">
+        <v>500</v>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G367" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I367" t="n">
+        <v>2366.762077273718</v>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K367" t="n">
+        <v>31.85819887323305</v>
+      </c>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M367" t="n">
+        <v>19117.03642711509</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>1</v>
+      </c>
+      <c r="B368" t="n">
+        <v>17</v>
+      </c>
+      <c r="C368" t="n">
+        <v>3</v>
+      </c>
+      <c r="D368" t="n">
+        <v>3600000</v>
+      </c>
+      <c r="E368" t="n">
+        <v>500</v>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G368" t="n">
+        <v>0.986</v>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I368" t="n">
+        <v>2766.055783689856</v>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K368" t="n">
+        <v>32.02090618014336</v>
+      </c>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M368" t="n">
+        <v>25461.90462833643</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>1</v>
+      </c>
+      <c r="B369" t="n">
+        <v>17</v>
+      </c>
+      <c r="C369" t="n">
+        <v>3</v>
+      </c>
+      <c r="D369" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="E369" t="n">
+        <v>500</v>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G369" t="n">
+        <v>0.992</v>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I369" t="n">
+        <v>2871.740602900768</v>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K369" t="n">
+        <v>31.86532167252153</v>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M369" t="n">
+        <v>24152.17337058485</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="n">
+        <v>1</v>
+      </c>
+      <c r="B370" t="n">
+        <v>17</v>
+      </c>
+      <c r="C370" t="n">
+        <v>3</v>
+      </c>
+      <c r="D370" t="n">
+        <v>600000</v>
+      </c>
+      <c r="E370" t="n">
+        <v>500</v>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G370" t="n">
+        <v>0.968</v>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I370" t="n">
+        <v>2855.6195996947</v>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K370" t="n">
+        <v>31.92887891642749</v>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M370" t="n">
+        <v>26063.27650208771</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="n">
+        <v>1</v>
+      </c>
+      <c r="B371" t="n">
+        <v>17</v>
+      </c>
+      <c r="C371" t="n">
+        <v>3</v>
+      </c>
+      <c r="D371" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E371" t="n">
+        <v>500</v>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G371" t="n">
+        <v>0.668</v>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I371" t="n">
+        <v>6701.265084237808</v>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K371" t="n">
+        <v>31.90760805486934</v>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M371" t="n">
+        <v>42245.01598630496</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Added self.mode data dumping and plotting state diagrams with CAD scans
</commit_message>
<xml_diff>
--- a/Tests/representative_network_1_sim_outputs.xlsx
+++ b/Tests/representative_network_1_sim_outputs.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-6030" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -124,14 +124,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -159,8 +159,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -190,7 +190,7 @@
             <v>2.2 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:srgbClr val="FF33CC"/>
               </a:solidFill>
@@ -201,7 +201,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -263,7 +263,7 @@
             <v>2.1 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:srgbClr val="7030A0"/>
               </a:solidFill>
@@ -274,7 +274,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -336,7 +336,7 @@
             <v>2.0 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:srgbClr val="00B0F0"/>
               </a:solidFill>
@@ -348,10 +348,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="00B0F0"/>
               </a:solidFill>
-              <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350" cap="flat" cmpd="sng" algn="ctr">
                 <a:solidFill>
                   <a:srgbClr val="00B0F0"/>
                 </a:solidFill>
@@ -417,7 +417,7 @@
             <v>1.9 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="accent6"/>
               </a:solidFill>
@@ -429,10 +429,10 @@
             <symbol val="diamond"/>
             <size val="6"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:schemeClr val="accent6"/>
               </a:solidFill>
-              <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350" cap="flat" cmpd="sng" algn="ctr">
                 <a:solidFill>
                   <a:schemeClr val="accent6"/>
                 </a:solidFill>
@@ -498,7 +498,7 @@
             <v>1.8 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
@@ -510,10 +510,10 @@
             <symbol val="triangle"/>
             <size val="6"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
-              <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350" cap="flat" cmpd="sng" algn="ctr">
                 <a:solidFill>
                   <a:schemeClr val="accent1"/>
                 </a:solidFill>
@@ -579,7 +579,7 @@
             <v>1.7 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="accent4">
                   <a:lumMod val="60000"/>
@@ -595,8 +595,8 @@
             <symbol val="x"/>
             <size val="6"/>
             <spPr>
-              <a:noFill/>
-              <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
                 <a:solidFill>
                   <a:srgbClr val="FF0000"/>
                 </a:solidFill>
@@ -677,9 +677,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -707,8 +707,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill/>
-            <a:ln>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -719,8 +719,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -732,9 +732,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -770,7 +770,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -785,9 +785,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -815,8 +815,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill/>
-            <a:ln>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -827,17 +827,17 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
             <a:prstDash val="solid"/>
             <a:round/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -878,16 +878,16 @@
       </layout>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -912,10 +912,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -930,14 +930,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -965,8 +965,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -996,7 +996,7 @@
             <v>1.0 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:srgbClr val="FF33CC"/>
               </a:solidFill>
@@ -1007,7 +1007,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1069,7 +1069,7 @@
             <v>0.9 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:srgbClr val="6600CC"/>
               </a:solidFill>
@@ -1080,7 +1080,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1142,7 +1142,7 @@
             <v>0.8 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="accent6"/>
               </a:solidFill>
@@ -1153,7 +1153,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1215,7 +1215,7 @@
             <v>0.7 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="accent1">
                   <a:lumMod val="75000"/>
@@ -1229,10 +1229,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:srgbClr val="0070C0"/>
               </a:solidFill>
-              <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350" cap="flat" cmpd="sng" algn="ctr">
                 <a:solidFill>
                   <a:srgbClr val="0070C0"/>
                 </a:solidFill>
@@ -1298,7 +1298,7 @@
             <v>0.6 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="accent2">
                   <a:lumMod val="75000"/>
@@ -1312,12 +1312,12 @@
             <symbol val="triangle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:schemeClr val="accent2">
                   <a:lumMod val="75000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350" cap="flat" cmpd="sng" algn="ctr">
                 <a:solidFill>
                   <a:schemeClr val="accent2">
                     <a:lumMod val="75000"/>
@@ -1385,7 +1385,7 @@
             <v>0.5 Seconds</v>
           </tx>
           <spPr>
-            <a:ln w="19050" cap="rnd" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="rnd" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="accent4"/>
               </a:solidFill>
@@ -1397,8 +1397,8 @@
             <symbol val="x"/>
             <size val="5"/>
             <spPr>
-              <a:noFill/>
-              <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700" cap="flat" cmpd="sng" algn="ctr">
                 <a:solidFill>
                   <a:schemeClr val="accent4"/>
                 </a:solidFill>
@@ -1479,9 +1479,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -1509,8 +1509,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill/>
-            <a:ln>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1521,8 +1521,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -1534,9 +1534,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1572,7 +1572,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -1587,9 +1587,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -1617,8 +1617,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill/>
-            <a:ln>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1629,17 +1629,17 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="6350" cap="flat" cmpd="sng" algn="ctr">
             <a:noFill/>
             <a:prstDash val="solid"/>
             <a:round/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1680,16 +1680,16 @@
       </layout>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
             <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -1714,10 +1714,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -1732,14 +1732,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -1767,8 +1767,8 @@
       </tx>
       <overlay val="0"/>
       <spPr>
-        <a:noFill/>
-        <a:ln>
+        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
@@ -1798,7 +1798,7 @@
             <v>With Traditional Flooding</v>
           </tx>
           <spPr>
-            <a:ln w="28575" cap="rnd">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="28575" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
@@ -1810,10 +1810,10 @@
             <symbol val="circle"/>
             <size val="5"/>
             <spPr>
-              <a:solidFill>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
-              <a:ln w="9525">
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
                 <a:solidFill>
                   <a:schemeClr val="accent1"/>
                 </a:solidFill>
@@ -1935,7 +1935,7 @@
             <v>With Routing</v>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1943,7 +1943,7 @@
             <symbol val="square"/>
             <size val="5"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -2111,9 +2111,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2144,8 +2144,8 @@
           </tx>
           <overlay val="0"/>
           <spPr>
-            <a:noFill/>
-            <a:ln>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2156,8 +2156,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -2169,9 +2169,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -2207,7 +2207,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -2222,9 +2222,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2262,8 +2262,8 @@
           </layout>
           <overlay val="0"/>
           <spPr>
-            <a:noFill/>
-            <a:ln>
+            <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2274,16 +2274,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill/>
-          <a:ln>
+          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -2328,10 +2328,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -2346,7 +2346,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>13</col>
@@ -2366,9 +2366,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2393,9 +2393,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2420,9 +2420,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2693,12 +2693,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N371"/>
+  <dimension ref="A1:N382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8" customWidth="1" min="3" max="3"/>
@@ -18847,8 +18847,547 @@
         <v>42245.01598630496</v>
       </c>
     </row>
+    <row r="372">
+      <c r="A372" t="n">
+        <v>1</v>
+      </c>
+      <c r="B372" t="n">
+        <v>17</v>
+      </c>
+      <c r="C372" t="n">
+        <v>3</v>
+      </c>
+      <c r="D372" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E372" t="n">
+        <v>100</v>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G372" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I372" t="n">
+        <v>3277.433681015776</v>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K372" t="n">
+        <v>33.34622008501901</v>
+      </c>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M372" t="n">
+        <v>15022.44048399839</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="n">
+        <v>1</v>
+      </c>
+      <c r="B373" t="n">
+        <v>17</v>
+      </c>
+      <c r="C373" t="n">
+        <v>3</v>
+      </c>
+      <c r="D373" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E373" t="n">
+        <v>100</v>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G373" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I373" t="n">
+        <v>3050.482189469526</v>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K373" t="n">
+        <v>32.58514194888994</v>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M373" t="n">
+        <v>13925.64766310493</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="n">
+        <v>1</v>
+      </c>
+      <c r="B374" t="n">
+        <v>17</v>
+      </c>
+      <c r="C374" t="n">
+        <v>3</v>
+      </c>
+      <c r="D374" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E374" t="n">
+        <v>100</v>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G374" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I374" t="n">
+        <v>3476.786842623643</v>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K374" t="n">
+        <v>32.38702146602736</v>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M374" t="n">
+        <v>20560.45402586949</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="n">
+        <v>1</v>
+      </c>
+      <c r="B375" t="n">
+        <v>17</v>
+      </c>
+      <c r="C375" t="n">
+        <v>3</v>
+      </c>
+      <c r="D375" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E375" t="n">
+        <v>100</v>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G375" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I375" t="n">
+        <v>2702.781333984933</v>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K375" t="n">
+        <v>32.6414845881518</v>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M375" t="n">
+        <v>20797.67314184736</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="n">
+        <v>1</v>
+      </c>
+      <c r="B376" t="n">
+        <v>17</v>
+      </c>
+      <c r="C376" t="n">
+        <v>3</v>
+      </c>
+      <c r="D376" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E376" t="n">
+        <v>100</v>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G376" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I376" t="n">
+        <v>3324.714877347291</v>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K376" t="n">
+        <v>33.58104137727059</v>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M376" t="n">
+        <v>25645.02759544184</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="n">
+        <v>1</v>
+      </c>
+      <c r="B377" t="n">
+        <v>17</v>
+      </c>
+      <c r="C377" t="n">
+        <v>3</v>
+      </c>
+      <c r="D377" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E377" t="n">
+        <v>100</v>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G377" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I377" t="n">
+        <v>2780.75551565079</v>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K377" t="n">
+        <v>31.99709318228997</v>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M377" t="n">
+        <v>21785.1189477602</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="n">
+        <v>1</v>
+      </c>
+      <c r="B378" t="n">
+        <v>17</v>
+      </c>
+      <c r="C378" t="n">
+        <v>3</v>
+      </c>
+      <c r="D378" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E378" t="n">
+        <v>100</v>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G378" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I378" t="n">
+        <v>1856.055164360395</v>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K378" t="n">
+        <v>32.10416393517517</v>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M378" t="n">
+        <v>9271.848588306224</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="n">
+        <v>1</v>
+      </c>
+      <c r="B379" t="n">
+        <v>17</v>
+      </c>
+      <c r="C379" t="n">
+        <v>3</v>
+      </c>
+      <c r="D379" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E379" t="n">
+        <v>100</v>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G379" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I379" t="n">
+        <v>2889.448891068846</v>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K379" t="n">
+        <v>32.41056588845095</v>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M379" t="n">
+        <v>24351.03240937949</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="n">
+        <v>1</v>
+      </c>
+      <c r="B380" t="n">
+        <v>17</v>
+      </c>
+      <c r="C380" t="n">
+        <v>3</v>
+      </c>
+      <c r="D380" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E380" t="n">
+        <v>100</v>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G380" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I380" t="n">
+        <v>2571.155592099362</v>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K380" t="n">
+        <v>32.14394230709877</v>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M380" t="n">
+        <v>13173.21727735689</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="n">
+        <v>1</v>
+      </c>
+      <c r="B381" t="n">
+        <v>17</v>
+      </c>
+      <c r="C381" t="n">
+        <v>3</v>
+      </c>
+      <c r="D381" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E381" t="n">
+        <v>100</v>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G381" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I381" t="n">
+        <v>3608.227121487305</v>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K381" t="n">
+        <v>32.40489910449833</v>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M381" t="n">
+        <v>24954.79982602177</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="n">
+        <v>1</v>
+      </c>
+      <c r="B382" t="n">
+        <v>17</v>
+      </c>
+      <c r="C382" t="n">
+        <v>3</v>
+      </c>
+      <c r="D382" t="n">
+        <v>360000</v>
+      </c>
+      <c r="E382" t="n">
+        <v>100</v>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>---&gt; DER:</t>
+        </is>
+      </c>
+      <c r="G382" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>---&gt; Avg Latency:</t>
+        </is>
+      </c>
+      <c r="I382" t="n">
+        <v>2821.853980816382</v>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>---&gt; Min Latency:</t>
+        </is>
+      </c>
+      <c r="K382" t="n">
+        <v>32.44769056420773</v>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>---&gt; Max Latency:</t>
+        </is>
+      </c>
+      <c r="M382" t="n">
+        <v>19156.87953486451</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added wor preamble time logging into a file
</commit_message>
<xml_diff>
--- a/Tests/representative_network_1_sim_outputs.xlsx
+++ b/Tests/representative_network_1_sim_outputs.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z5440292_ad_unsw_edu_au/Documents/MyPhD-Workspace/Codes/LoRaMeshSimulator-V3/Tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_DD8ED4682BBE59FF2170FBD0962F65E38DA02FD4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2889BB0F-23B2-4E6F-B0AE-925FCE83F709}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_DD8ED4682BBE59FF2170FBD0962F65E38DA02FD4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2D01965-3FDB-45EB-ABEC-9D0EAE235716}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-6030" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-12060" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -2397,6 +2400,720 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.11229372820501815"/>
+          <c:y val="5.8728368847519613E-2"/>
+          <c:w val="0.78140634910052964"/>
+          <c:h val="0.78030103207737567"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>with sleep mode</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>[1]Sheet1!$AG$2:$AG$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0.70833333333333337</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.4166666666666667</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.8333333333333335</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.666666666666667</c:v>
+                </c:pt>
+                <c:pt idx="4" formatCode="General">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="General">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="6" formatCode="General">
+                  <c:v>102</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>[1]Sheet1!$X$2:$X$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>2.2281316009388041E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.6867033718468051E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.8077359154637877E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.9780470832497677E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.17289327659562509</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.32398987188198453</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.83039944910561592</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3DC7-40ED-B4D3-75E92DD658D1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1570810751"/>
+        <c:axId val="1570811231"/>
+      </c:lineChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>without sleep mode</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="triangle"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>[1]Sheet1!$AG$20:$AG$26</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>0.70833333333333337</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.4166666666666667</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.8333333333333335</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5.666666666666667</c:v>
+                </c:pt>
+                <c:pt idx="4" formatCode="General">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="General">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="6" formatCode="General">
+                  <c:v>102</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>[1]Sheet1!$X$10:$X$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>13.562706692476439</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>13.58172066553848</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>13.86073945495365</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>13.92250861967292</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>13.924694683487679</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>13.928716656420359</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>13.97474619678326</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-3DC7-40ED-B4D3-75E92DD658D1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="361892976"/>
+        <c:axId val="361895856"/>
+        <c:extLst>
+          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+            <c15:filteredLineSeries>
+              <c15:ser>
+                <c:idx val="2"/>
+                <c:order val="2"/>
+                <c:tx>
+                  <c:v>with sleep mode (unsync)</c:v>
+                </c:tx>
+                <c:spPr>
+                  <a:ln>
+                    <a:prstDash val="solid"/>
+                  </a:ln>
+                </c:spPr>
+                <c:marker>
+                  <c:symbol val="none"/>
+                </c:marker>
+                <c:cat>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[1]Sheet1!$AG$20:$AG$26</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>0.00</c:formatCode>
+                      <c:ptCount val="7"/>
+                      <c:pt idx="0">
+                        <c:v>0.70833333333333337</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>1.4166666666666667</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>2.8333333333333335</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>5.666666666666667</c:v>
+                      </c:pt>
+                      <c:pt idx="4" formatCode="General">
+                        <c:v>17</c:v>
+                      </c:pt>
+                      <c:pt idx="5" formatCode="General">
+                        <c:v>34</c:v>
+                      </c:pt>
+                      <c:pt idx="6" formatCode="General">
+                        <c:v>102</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:cat>
+                <c:val>
+                  <c:numRef>
+                    <c:extLst>
+                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
+                        <c15:formulaRef>
+                          <c15:sqref>[1]Sheet1!$X$20:$X$26</c15:sqref>
+                        </c15:formulaRef>
+                      </c:ext>
+                    </c:extLst>
+                    <c:numCache>
+                      <c:formatCode>General</c:formatCode>
+                      <c:ptCount val="7"/>
+                      <c:pt idx="0">
+                        <c:v>2.274879227113405E-2</c:v>
+                      </c:pt>
+                      <c:pt idx="1">
+                        <c:v>2.749108937624585E-2</c:v>
+                      </c:pt>
+                      <c:pt idx="2">
+                        <c:v>4.2946770556080677E-2</c:v>
+                      </c:pt>
+                      <c:pt idx="3">
+                        <c:v>7.6705999954475565E-2</c:v>
+                      </c:pt>
+                      <c:pt idx="4">
+                        <c:v>0.18520095608619419</c:v>
+                      </c:pt>
+                      <c:pt idx="5">
+                        <c:v>0.3253889721440108</c:v>
+                      </c:pt>
+                      <c:pt idx="6">
+                        <c:v>1.257376388966682</c:v>
+                      </c:pt>
+                    </c:numCache>
+                  </c:numRef>
+                </c:val>
+                <c:smooth val="0"/>
+                <c:extLst>
+                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                    <c16:uniqueId val="{00000002-3DC7-40ED-B4D3-75E92DD658D1}"/>
+                  </c:ext>
+                </c:extLst>
+              </c15:ser>
+            </c15:filteredLineSeries>
+          </c:ext>
+        </c:extLst>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1570810751"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="900"/>
+                  <a:t>Network's</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="900" baseline="0"/>
+                  <a:t> Packet Input Rate</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="900"/>
+                  <a:t> (per hour)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:prstDash val="solid"/>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1570811231"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1570811231"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1.4"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="900">
+                    <a:solidFill>
+                      <a:schemeClr val="accent1"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Avg. Power Usage by a Repeater per hr (mAh)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1570810751"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="361892976"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="361895856"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="361895856"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="14"/>
+          <c:min val="12"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="r"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="accent2"/>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Avg. Power Usage by a Repeater per hr (mAh)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="361892976"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="0.5"/>
+        <c:minorUnit val="0.1"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.15612889615622935"/>
+          <c:y val="0.47311898523999557"/>
+          <c:w val="0.3524913801802822"/>
+          <c:h val="0.14169312312084789"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -2507,7 +3224,213 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>270</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>155662</xdr:colOff>
+      <xdr:row>286</xdr:row>
+      <xdr:rowOff>119566</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{038F0B33-5D69-4C2B-94D5-409D7AA5AE63}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Sheet1"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="2">
+          <cell r="X2">
+            <v>2.2281316009388041E-2</v>
+          </cell>
+          <cell r="AG2">
+            <v>0.70833333333333337</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="X3">
+            <v>2.6867033718468051E-2</v>
+          </cell>
+          <cell r="AG3">
+            <v>1.4166666666666667</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="X4">
+            <v>3.8077359154637877E-2</v>
+          </cell>
+          <cell r="AG4">
+            <v>2.8333333333333335</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="X5">
+            <v>5.9780470832497677E-2</v>
+          </cell>
+          <cell r="AG5">
+            <v>5.666666666666667</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="X6">
+            <v>0.17289327659562509</v>
+          </cell>
+          <cell r="AG6">
+            <v>17</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="X7">
+            <v>0.32398987188198453</v>
+          </cell>
+          <cell r="AG7">
+            <v>34</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="X8">
+            <v>0.83039944910561592</v>
+          </cell>
+          <cell r="AG8">
+            <v>102</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="X10">
+            <v>13.562706692476439</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="X11">
+            <v>13.58172066553848</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="X12">
+            <v>13.86073945495365</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="X13">
+            <v>13.92250861967292</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="X14">
+            <v>13.924694683487679</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="X15">
+            <v>13.928716656420359</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="X16">
+            <v>13.97474619678326</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="X20">
+            <v>2.274879227113405E-2</v>
+          </cell>
+          <cell r="AG20">
+            <v>0.70833333333333337</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="X21">
+            <v>2.749108937624585E-2</v>
+          </cell>
+          <cell r="AG21">
+            <v>1.4166666666666667</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="X22">
+            <v>4.2946770556080677E-2</v>
+          </cell>
+          <cell r="AG22">
+            <v>2.8333333333333335</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="X23">
+            <v>7.6705999954475565E-2</v>
+          </cell>
+          <cell r="AG23">
+            <v>5.666666666666667</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="X24">
+            <v>0.18520095608619419</v>
+          </cell>
+          <cell r="AG24">
+            <v>17</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="X25">
+            <v>0.3253889721440108</v>
+          </cell>
+          <cell r="AG25">
+            <v>34</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="X26">
+            <v>1.257376388966682</v>
+          </cell>
+          <cell r="AG26">
+            <v>102</v>
+          </cell>
+        </row>
+      </sheetData>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>